<commit_message>
Updated FRA_grids_syn_5 model - 2025-10-14 12:02
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_FRA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F495BBDD-525A-4A52-936E-49F0DBCEF378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F059B5D-772D-4D34-AAFF-D1EFC55797C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9526,7 +9526,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C872E89A-FA3C-41F8-9F84-FC0C7458E08A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FA0CB6-E13C-427F-9256-5D579CDA5912}">
   <dimension ref="B9:H170"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12764,7 +12764,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{215CF96C-0DA9-446D-B7E7-27FC1C712764}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{846B33C2-0CA6-43CF-802A-80674A1EC351}">
   <dimension ref="B9:L170"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated FRA_grids_syn_5 model - 2025-10-14 12:20
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_FRA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F059B5D-772D-4D34-AAFF-D1EFC55797C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{40B68629-E1C6-41FA-8E31-B21E725D226D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9526,7 +9526,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FA0CB6-E13C-427F-9256-5D579CDA5912}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45A7165D-F6FD-4FA3-B741-8034160C4926}">
   <dimension ref="B9:H170"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12764,7 +12764,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{846B33C2-0CA6-43CF-802A-80674A1EC351}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0144EDBC-5860-4E6D-872D-2BAF97DADF60}">
   <dimension ref="B9:L170"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated FRA_grids_syn_5 model - 2025-10-14 12:28
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_FRA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40B68629-E1C6-41FA-8E31-B21E725D226D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9BC146E-5F08-4E68-A9EB-E9010E165D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9526,7 +9526,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45A7165D-F6FD-4FA3-B741-8034160C4926}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E0FA78-D8EE-4A92-8421-C0315877F234}">
   <dimension ref="B9:H170"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12764,7 +12764,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0144EDBC-5860-4E6D-872D-2BAF97DADF60}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0839EA73-9558-473A-885A-9F369F870C0B}">
   <dimension ref="B9:L170"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated FRA_grids_syn_5 model - 2025-10-14 13:49
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_FRA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9BC146E-5F08-4E68-A9EB-E9010E165D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{28DBDE52-3814-45A1-8391-EEE61D3EC953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1103" yWindow="1103" windowWidth="21600" windowHeight="12682" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -9526,7 +9526,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E0FA78-D8EE-4A92-8421-C0315877F234}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40983669-49E3-4708-95CD-15DD69C163D3}">
   <dimension ref="B9:H170"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12764,7 +12764,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0839EA73-9558-473A-885A-9F369F870C0B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39318F7D-675B-4CC8-B123-5BFF23089799}">
   <dimension ref="B9:L170"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>